<commit_message>
feat: improve Bosch resolver with family tech sheet inheritance and JPG export
</commit_message>
<xml_diff>
--- a/data/input/bosch.xlsx
+++ b/data/input/bosch.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nas18\OneDrive\Escritorio\Soler Teselen\supplier-scraper\data\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://solerteselen-my.sharepoint.com/personal/jcvega_solerteselen_cat/Documents/Escritorio/jean/Codigo Soler Teselen/supplier-scrapi/data/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92CAE6DD-321F-4BC3-8E8F-9EC18063EC92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{92CAE6DD-321F-4BC3-8E8F-9EC18063EC92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E6515864-04BA-4C4D-8974-FAE2CD028F10}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="18855" windowHeight="14310" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="74">
   <si>
     <t>nombre</t>
   </si>
@@ -43,14 +43,226 @@
   </si>
   <si>
     <t>referencia</t>
+  </si>
+  <si>
+    <t>BOSCH CALDERA CONDENSACIÓ GC4300I W 24/25 NAT.</t>
+  </si>
+  <si>
+    <t>7731200602</t>
+  </si>
+  <si>
+    <t>BOSCH CALDERA CONDENSACIÓ GC6000 W 25/28 NAT.</t>
+  </si>
+  <si>
+    <t>7731200597</t>
+  </si>
+  <si>
+    <t>BOSCH CALD MUR.CONDCN.MXT.C4300I W 24/30 GN 24KW 710X400X300</t>
+  </si>
+  <si>
+    <t>7731200600</t>
+  </si>
+  <si>
+    <t>BOSCH ESCALFADOR GAS BAIX NOX THERM 6600 S 12 D31 BUTÀ 60/10</t>
+  </si>
+  <si>
+    <t>7731200811</t>
+  </si>
+  <si>
+    <t>BOSCH ESCALFADOR GAS BAIX NOX THERM 6600 S 12 D23 NAT 60/100</t>
+  </si>
+  <si>
+    <t>7731200810</t>
+  </si>
+  <si>
+    <t>BOSCH ESCALFADOR GAS BAIX NOX THERM 6600 S 15 D31 BUTÀ 60/10</t>
+  </si>
+  <si>
+    <t>7731200813</t>
+  </si>
+  <si>
+    <t>BOSCH ESCALFADOR GAS BAIX NOX THERM 6600 S 15 D23 NAT 60/100</t>
+  </si>
+  <si>
+    <t>7731200812</t>
+  </si>
+  <si>
+    <t>BOSCH ESCALFADOR GAS BAIX NOX THERM 6600 S 17 D31 BUTÀ 60/10</t>
+  </si>
+  <si>
+    <t>7731200815</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR2000T VERTICAL  30 B</t>
+  </si>
+  <si>
+    <t>7736503346</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR2000T VERTICAL  50 B</t>
+  </si>
+  <si>
+    <t>7736503347</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR2000T VERTICAL  80 B</t>
+  </si>
+  <si>
+    <t>7736503349</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR2000T VERTICAL 100 B</t>
+  </si>
+  <si>
+    <t>7736503351</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR2000T VERTICAL 120 B</t>
+  </si>
+  <si>
+    <t>7736503353</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR2000T VERTICAL SLIM  50 SB</t>
+  </si>
+  <si>
+    <t>7736506818</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR2000T VERTICAL SLIM  80 SB</t>
+  </si>
+  <si>
+    <t>7736506819</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR1001T VERTICAL 150 B</t>
+  </si>
+  <si>
+    <t>7736506470</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR1001T VERTICAL 200 B</t>
+  </si>
+  <si>
+    <t>7736506475</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR1001T VERTICAL 300 T</t>
+  </si>
+  <si>
+    <t>7736506480</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR2102T VERTICAL 35 B</t>
+  </si>
+  <si>
+    <t>7724000062</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR2102T REVERSIBLE  50 RB</t>
+  </si>
+  <si>
+    <t>7724000063</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR2102T REVERSIBLE  80 RB</t>
+  </si>
+  <si>
+    <t>7724000064</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR2102T REVERSIBLE 100 RB</t>
+  </si>
+  <si>
+    <t>7724000065</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR2102T REVERSIBLE 120 RB</t>
+  </si>
+  <si>
+    <t>7724000066</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR2102T REVERSIBLE 150 RB</t>
+  </si>
+  <si>
+    <t>7724000067</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR4101T VERTICAL DISPLAY  50 DEBS</t>
+  </si>
+  <si>
+    <t>7736507539</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR4101T VERTICAL DISPLAY  80 DEB</t>
+  </si>
+  <si>
+    <t>7736507540</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR4101T VERTICAL DISPLAY  100 DEB</t>
+  </si>
+  <si>
+    <t>7736507541</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR4101T VERTICAL DISPLAY  120 DEB</t>
+  </si>
+  <si>
+    <t>7736507556</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR7501T PLA REVERSIBLE DIGITAL 50</t>
+  </si>
+  <si>
+    <t>7736507274</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR7501T PLA REVERSIBLE DIGITAL 70</t>
+  </si>
+  <si>
+    <t>7736507275</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR7501T PLA REVERSIBLE DIGITAL 80</t>
+  </si>
+  <si>
+    <t>7736507276</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR7501T PLA REVERSIBLE DIGITAL 100</t>
+  </si>
+  <si>
+    <t>7736507277</t>
+  </si>
+  <si>
+    <t>BOSCH TERMOS ELECTRIC TR7501T PLA REVERSIBLE DIGITAL 120</t>
+  </si>
+  <si>
+    <t>7736507441</t>
+  </si>
+  <si>
+    <t>BOSCH TERMO ELÉC. TRONIC 7101 T VERTICAL TR7101T 120 DE</t>
+  </si>
+  <si>
+    <t>7736507555</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -80,7 +292,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -361,7 +573,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="62.140625" bestFit="1" customWidth="1"/>
@@ -378,19 +590,294 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>2</v>
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>3</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B11" t="s">
         <v>4</v>
       </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>48</v>
+      </c>
+      <c r="B25" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>54</v>
+      </c>
+      <c r="B28" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>56</v>
+      </c>
+      <c r="B29" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>58</v>
+      </c>
+      <c r="B30" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>60</v>
+      </c>
+      <c r="B31" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>62</v>
+      </c>
+      <c r="B32" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B33" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>66</v>
+      </c>
+      <c r="B34" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>68</v>
+      </c>
+      <c r="B35" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>70</v>
+      </c>
+      <c r="B36" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>72</v>
+      </c>
+      <c r="B37" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F42" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>